<commit_message>
Update importExport.py to current version from branch feature/Dyler.
</commit_message>
<xml_diff>
--- a/data/example/Power_Parameters.xlsx
+++ b/data/example/Power_Parameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo\data\example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC4CDDB-9480-4559-A267-496F079188FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD86268-C279-4592-95AE-389334B73F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33915" yWindow="-21810" windowWidth="38640" windowHeight="21120" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Parameters" sheetId="121" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="93">
   <si>
     <t>[p.u.]</t>
   </si>
@@ -342,13 +342,7 @@
     <t>Format:</t>
   </si>
   <si>
-    <t>Intra-Day Storage constraint type for edge timesteps</t>
-  </si>
-  <si>
-    <t>pReprPeriodEdgeHandlingIntraDayStorage</t>
-  </si>
-  <si>
-    <t>v0.2.0</t>
+    <t>v0.1.0</t>
   </si>
 </sst>
 </file>
@@ -577,21 +571,7 @@
     <cellStyle name="Standard 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
     <cellStyle name="Standard 4" xfId="7" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
   </cellStyles>
-  <dxfs count="34">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFB90135"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF4E9C49"/>
-      </font>
-    </dxf>
+  <dxfs count="32">
     <dxf>
       <font>
         <b/>
@@ -1133,7 +1113,7 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="B1:H79"/>
+  <dimension ref="B1:H76"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" style="1" customWidth="1"/>
@@ -1157,7 +1137,7 @@
         <v>91</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1369,7 +1349,7 @@
         <v>58</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>82</v>
@@ -1729,162 +1709,132 @@
         <v>71</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C78" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="79" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C6 C14:C28">
-    <cfRule type="cellIs" dxfId="33" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="39" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="40" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8:C9">
-    <cfRule type="cellIs" dxfId="31" priority="101" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="99" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="102" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="100" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="cellIs" dxfId="29" priority="99" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="97" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="98" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C31">
-    <cfRule type="cellIs" dxfId="27" priority="111" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="109" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="112" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="110" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34">
-    <cfRule type="cellIs" dxfId="25" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="87" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="90" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="88" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C37 C40">
-    <cfRule type="cellIs" dxfId="23" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="85" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="88" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="86" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43">
-    <cfRule type="cellIs" dxfId="21" priority="85" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="83" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="84" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46">
-    <cfRule type="cellIs" dxfId="19" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="81" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="82" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49">
-    <cfRule type="cellIs" dxfId="17" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="79" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="80" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C53 C56">
-    <cfRule type="cellIs" dxfId="15" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="43" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="44" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C60:C61">
-    <cfRule type="cellIs" dxfId="13" priority="95" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="93" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="94" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C63:C64">
-    <cfRule type="cellIs" dxfId="11" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="31" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="32" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C66:C67">
-    <cfRule type="cellIs" dxfId="9" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="27" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="28" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C69:C70">
-    <cfRule type="cellIs" dxfId="7" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C73">
-    <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="21" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="22" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C76">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C79">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1893,7 +1843,7 @@
       <formula1>"No, Yes"</formula1>
     </dataValidation>
     <dataValidation showInputMessage="1" showErrorMessage="1" sqref="C9 C12 C61 C64 C67 C70 C15:C28" xr:uid="{87C6F772-FD4B-9449-B9E7-DA0FF0A031BB}"/>
-    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C60 C46 C63 C66 C69 C73 C76 C79" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
+    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C60 C46 C63 C66 C69 C73 C76" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>